<commit_message>
NPB自動更新(2軍): 2026-08-28 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/2軍/公式戦/games/datamart/2026-08-28.xlsx
+++ b/data/プロ野球/2026年/2軍/公式戦/games/datamart/2026-08-28.xlsx
@@ -57741,17 +57741,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ガルシア</t>
+          <t>石塚 綜一郎</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>阪神</t>
+          <t>ソフトバンク</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5回表に左中間へ逆転2ランホームランを放ち、試合の流れを大きく変えた。</t>
+          <t>7回裏にダメ押しとなる本塁打を放ち、3打点を挙げて勝利を決定づけた。</t>
         </is>
       </c>
     </row>
@@ -57766,17 +57766,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>池田 陵真</t>
+          <t>川原田 純平</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>オリックス</t>
+          <t>巨人</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1回裏に先制2ランホームラン、さらに3回裏には勝ち越しタイムリーを放ち活躍。</t>
+          <t>7回表に均衡を破る先制タイムリーヒットを放ち、チームの勝利に貢献した。</t>
         </is>
       </c>
     </row>
@@ -57791,7 +57791,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>石塚 綜一郎</t>
+          <t>イヒネ イツア</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -57801,7 +57801,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7回裏にダメ押しのホームランを放ち、チームの勝利を決定づける一打となった。</t>
+          <t>5回裏に勝ち越し打、7回裏にもタイムリーを放ち、複数打点で勝利に貢献。</t>
         </is>
       </c>
     </row>
@@ -57816,17 +57816,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>川原田 純平</t>
+          <t>ガルシア</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>巨人</t>
+          <t>阪神</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7回表に三塁走者を返す先制タイムリーヒットを放ち、チームの得点に貢献した。</t>
+          <t>5回表に試合をひっくり返す逆転2ランホームランを放ち、猛打賞の活躍を見せた。</t>
         </is>
       </c>
     </row>
@@ -57841,17 +57841,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>イヒネ イツア</t>
+          <t>池田 陵真</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ソフトバンク</t>
+          <t>オリックス</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>5回裏に勝ち越しタイムリーヒットを放ち、試合の主導権を握る重要な一打となった。</t>
+          <t>1回裏に先制2ラン、3回裏に勝ち越し打と、重要な局面で活躍した。</t>
         </is>
       </c>
     </row>
@@ -57876,7 +57876,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3安打猛打賞を記録し、5回裏にはタイムリーツーベースでチームの得点に貢献。</t>
+          <t>5回裏にタイムリーツーベースを放ち、猛打賞を記録して打線を牽引した。</t>
         </is>
       </c>
     </row>

</xml_diff>